<commit_message>
feat: Enhance text extraction and comparison pipeline
- Introduced page markers in markdown output to track origin of text blocks.
- Implemented functions to parse and strip page markers for improved text analysis.
- Added canonical markdown path retrieval to avoid redundant Docling runs.
- Updated text extraction and comparison logic to utilize new page indexing.
- Improved error handling and logging for markdown processing.
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changements détectés" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -579,8 +579,8 @@
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>La note de bas de page n-1 a été ajoutée dans le tableau des échéances contractuelles des actifs financiers au T2 2025.
-Cette note précise l'impact de l'acquisition de CWB par la Banque, en indiquant que les résultats de CWB ont été consolidés à partir de la date de clôture, ce qui a affecté les soldes au 30 avril 2025. Cette information est cruciale pour comprendre les variations des soldes financiers présentés dans le tableau, car elle introduit un changement structurel dans la composition des actifs de la Banque.
-Il s'agit d'une divulgation importante qui pourrait avoir des implications sur les ratios prudentiels et la perception des investisseurs quant à la solidité financière de la Banque. L'analyste devrait confirmer l'intégration correcte de ces résultats dans les états financiers consolidés et s'assurer que toutes les implications réglementaires, notamment celles liées aux exigences de Bâle III, sont bien respectées.</t>
+Cette note précise l'impact de l'acquisition de CWB par la Banque, en indiquant que les résultats de CWB ont été consolidés à partir de la date de clôture, ce qui a affecté les soldes au 30 avril 2025. Cette information est cruciale car elle peut influencer la perception des investisseurs et des régulateurs sur la solidité financière de la Banque, notamment en ce qui concerne les ratios de capital et de liquidité. L'acquisition pourrait également avoir des implications sur les exigences de fonds propres selon les normes de Bâle III, en raison de l'intégration de nouveaux actifs et passifs.
+Il s'agit d'une divulgation importante qui pourrait avoir des implications structurelles sur l'analyse des états financiers de la Banque. L'analyste devrait confirmer l'intégration correcte de cette acquisition dans les autres sections du rapport financier et s'assurer que toutes les implications réglementaires ont été correctement adressées.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -632,9 +632,9 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Risques émergents – Hausse et incertitude des droits de douane et des restrictions sur les échanges commerciaux" a été ajouté dans le tableau de gestion des risques au T2 2025. Cet ajout remplace l'indicateur précédent qui portait sur les droits de douane sur les importations, en élargissant le champ pour inclure l'incertitude et les restrictions commerciales.
-Ce changement reflète une mise à jour des risques émergents liés aux échanges commerciaux, qui peuvent avoir un impact significatif sur les opérations bancaires internationales et la gestion des risques de crédit. Les incertitudes commerciales peuvent affecter les prévisions économiques et les stratégies de couverture des risques, ce qui est crucial pour les institutions financières.
-Il s'agit d'une mise à jour ordinaire qui reflète l'évolution des conditions économiques mondiales. L'analyste devrait confirmer que cette mise à jour est alignée avec les autres sections du rapport sur les risques et qu'elle est cohérente avec les analyses économiques actuelles.</t>
+          <t>L'indicateur "Risques émergents – Hausse et incertitude des droits de douane et des restrictions sur les échanges commerciaux" a été ajouté dans le tableau de gestion des risques au T2 2025, alors qu'il n'était pas présent au T1 2025.
+Cet ajout reflète une attention accrue aux risques liés aux fluctuations des droits de douane et aux restrictions commerciales, qui peuvent avoir un impact significatif sur les opérations bancaires internationales et la gestion des risques de crédit. Les institutions financières doivent surveiller ces évolutions pour ajuster leurs stratégies de couverture et de gestion des risques, conformément aux lignes directrices prudentielles.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cet ajout est aligné avec les autres sections du rapport sur les risques émergents et évaluer l'impact potentiel sur les stratégies de gestion des risques de l'institution.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -686,9 +686,9 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Risques émergents – Droits de douane sur les importations" a été retiré du tableau de gestion des risques au T2 2025. Cet indicateur a été remplacé par un nouveau qui couvre un champ plus large incluant l'incertitude et les restrictions commerciales.
-La suppression de cet indicateur spécifique peut refléter un changement dans la manière dont la banque évalue et communique les risques liés aux échanges commerciaux. Cela peut avoir des implications sur la gestion des risques de crédit et la planification stratégique, car les droits de douane et les restrictions commerciales peuvent influencer les flux commerciaux et les relations économiques internationales.
-Il s'agit d'une mise à jour ordinaire qui s'inscrit dans l'évolution des pratiques de gestion des risques. L'analyste devrait vérifier que cette suppression est bien documentée et que les nouvelles informations fournies sont cohérentes avec les autres analyses de risques du rapport.</t>
+          <t>L'indicateur "Risques émergents – Droits de douane sur les importations" a été retiré du tableau de gestion des risques au T2 2025, alors qu'il était présent au T1 2025.
+Ce retrait peut indiquer un changement dans la focalisation des risques émergents, passant d'une attention spécifique aux droits de douane sur les importations à une perspective plus large incluant les incertitudes et restrictions commerciales. Cela peut refléter une réévaluation des priorités en matière de gestion des risques, en réponse à des évolutions économiques ou politiques récentes.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier si ce retrait est compensé par d'autres indicateurs ou sections du rapport, et évaluer l'impact sur la stratégie globale de gestion des risques de l'institution.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -742,7 +742,7 @@
         <is>
           <t>L'indicateur "Série 47" a été ajouté dans le tableau des actions privilégiées et autres instruments de capitaux propres au T2 2025, alors qu'il était absent au T1 2025.
 Cet ajout pourrait indiquer l'émission d'une nouvelle série d'actions privilégiées, ce qui peut avoir un impact sur la structure du capital de la banque. Les actions privilégiées sont souvent utilisées pour renforcer les fonds propres de catégorie 1, conformément aux exigences de Bâle III et aux lignes directrices du BSIF.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer l'émission de cette nouvelle série et évaluer son impact sur les ratios de fonds propres.</t>
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer l'émission de cette nouvelle série et s'assurer que les informations sont cohérentes avec les autres divulgations financières.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-19T00:12:24.935014+00:00</t>
+          <t>2026-04-23T18:57:41.194006+00:00</t>
         </is>
       </c>
     </row>
@@ -807,8 +807,8 @@
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>L'indicateur "Série 49" a été ajouté dans le tableau des actions privilégiées et autres instruments de capitaux propres au T2 2025, alors qu'il était absent au T1 2025.
-Cet ajout pourrait indiquer l'émission d'une nouvelle série d'actions privilégiées, ce qui peut avoir un impact sur la structure du capital de la banque. Les actions privilégiées sont souvent utilisées pour renforcer les fonds propres de catégorie 1, conformément aux exigences de Bâle III et aux lignes directrices du BSIF.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer l'émission de cette nouvelle série et évaluer son impact sur les ratios de fonds propres.</t>
+L'ajout de cette série suggère une nouvelle émission d'actions privilégiées, ce qui peut influencer la composition des fonds propres de la banque. Les actions privilégiées jouent un rôle clé dans le renforcement des ratios de fonds propres, en ligne avec les exigences réglementaires de Bâle III.
+Il s'agit d'une mise à jour structurelle significative. L'analyste devrait vérifier l'exactitude de cette nouvelle émission et son impact sur les ratios de fonds propres.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -861,8 +861,8 @@
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>L'indicateur "Série 32" a été retiré du tableau des actions privilégiées et autres instruments de capitaux propres au T2 2025, alors qu'il était présent au T1 2025.
-La suppression de cette série pourrait indiquer le rachat ou l'annulation de cette série d'actions privilégiées, ce qui peut affecter la composition des fonds propres de la banque. Les actions privilégiées jouent un rôle clé dans le calcul des ratios de fonds propres de catégorie 1, en lien avec les exigences de Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier les raisons de cette suppression et son impact sur les ratios de fonds propres.</t>
+La suppression de cette série peut indiquer le rachat ou l'annulation de cette émission d'actions privilégiées, ce qui pourrait affecter la structure du capital de la banque. Les actions privilégiées sont essentielles pour maintenir les ratios de fonds propres requis par Bâle III.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer la raison de cette suppression et évaluer son impact sur les ratios de fonds propres et la conformité réglementaire.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -914,9 +914,9 @@
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>La note de bas de page n°3 a été supprimée dans le tableau de gestion du capital réglementaire, du ratio de levier et du TLAC entre le T1 2025 et le T2 2025. Cette note indiquait que les données au 31 janvier 2025 prenaient en compte le rachat d’actions privilégiées série 32 effectué le 17 février 2025.
-L'absence de cette note dans le rapport du T2 2025 pourrait avoir un impact sur la compréhension des ajustements de capital pour les parties prenantes. Le rachat d'actions privilégiées peut influencer les fonds propres de catégorie 1 et, par conséquent, les ratios de capital réglementaire. Selon les lignes directrices de Bâle III et les exigences du BSIF, les institutions financières doivent divulguer les événements significatifs qui affectent leur capital réglementaire.
-Il s'agit d'une mise à jour structurelle qui pourrait refléter un changement dans la manière dont les événements postérieurs à la date de clôture sont rapportés. L'analyste devrait confirmer que l'impact de ce rachat est correctement intégré dans les chiffres présentés et que l'absence de la note ne compromet pas la transparence des informations fournies.</t>
+          <t>La note de bas de page n°3 a été supprimée dans le tableau de gestion du capital réglementaire, du ratio de levier et du TLAC. Cette note faisait référence à l'impact du rachat d'actions privilégiées série 32 sur les données au 31 janvier 2025.
+L'absence de cette note dans le rapport actuel pourrait indiquer que l'effet de ce rachat n'est plus pertinent pour la période actuelle ou que l'information a été intégrée ailleurs dans le rapport. Cela pourrait avoir un impact sur la compréhension des ajustements de capital et des ratios de fonds propres, notamment si ces ajustements influencent les calculs de Bâle III ou les exigences du BSIF.
+Il s'agit potentiellement d'une mise à jour structurelle. L'analyste devrait confirmer si l'impact du rachat d'actions a été traité différemment dans le rapport actuel ou s'il est devenu obsolète. Une vérification de la cohérence avec d'autres sections du rapport est recommandée.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -925,9 +925,21 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23T18:59:00.240659+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -968,9 +980,9 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>La note de bas de page n°4 a été supprimée dans le tableau des exigences réglementaires de ratios des fonds propres, de levier et TLAC au T2 2025.
-Cette note indiquait que les ratios au 31 janvier 2025 prenaient en compte le rachat d’actions privilégiées série 32 effectué le 17 février 2025. La suppression de cette note pourrait signifier que cet événement n'est plus pertinent pour le calcul des ratios actuels ou que l'impact de cet événement a été entièrement intégré dans les chiffres actuels. Cela pourrait avoir des implications sur la transparence des divulgations financières, car les investisseurs et les régulateurs s'attendent à une explication claire des événements significatifs qui influencent les ratios de capital.
-Il s'agit d'une mise à jour potentiellement significative qui pourrait affecter la compréhension des ratios de capital par les parties prenantes. L'analyste devrait confirmer si cette suppression est due à l'intégration complète de l'impact de l'événement ou si d'autres facteurs ont influencé cette décision. Une vérification de la cohérence avec d'autres sections du rapport est recommandée.</t>
+          <t>La note de bas de page n°4 a été supprimée dans le tableau des exigences réglementaires de ratios des fonds propres, de levier et TLAC au T2 2025. Cette note indiquait que les ratios au 31 janvier 2025 prenaient en compte le rachat d’actions privilégiées série 32 effectué le 17 février 2025.
+L'absence de cette note dans le rapport actuel pourrait avoir un impact sur la transparence des informations fournies aux investisseurs et aux régulateurs. En effet, le rachat d'actions privilégiées peut influencer les ratios de fonds propres, et son omission pourrait masquer des variations importantes dans les calculs des ratios prudentiels. Selon les lignes directrices du BSIF, toute modification significative des éléments de fonds propres doit être clairement divulguée pour assurer la conformité avec les exigences de Bâle III.
+Il s'agit d'une mise à jour potentiellement significative qui pourrait indiquer un changement dans la manière dont les événements postérieurs sont pris en compte dans les calculs des ratios. L'analyste devrait confirmer si cette omission est intentionnelle et si elle est conforme aux pratiques de divulgation actuelles. Une investigation plus approfondie est recommandée pour s'assurer que toutes les informations pertinentes sont correctement communiquées.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1023,8 +1035,8 @@
       <c r="I10" s="2" t="inlineStr">
         <is>
           <t>L'indicateur "Risque de marché – Acquisitions et cessions" a été ajouté dans le tableau de gestion du capital au T2 2025, alors qu'il était absent au T1 2025.
-Cet ajout permet de mieux comprendre l'impact des acquisitions et cessions sur le risque de marché, ce qui est crucial pour évaluer les changements dans le profil de risque global de l'institution. Cela pourrait être lié à des changements dans la stratégie d'investissement ou à des exigences accrues de divulgation.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait s'assurer que cette nouvelle information est intégrée de manière cohérente avec les autres indicateurs de risque et qu'elle est conforme aux normes de divulgation.</t>
+Cet ajout permet de mieux isoler l'impact des acquisitions et cessions sur le risque de marché, ce qui est crucial pour l'évaluation des risques et la planification stratégique. Cela pourrait être lié à des changements dans la structure de l'entreprise ou à des exigences de divulgation accrues.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait s'assurer que cette nouvelle catégorie est justifiée par des changements dans les opérations ou les exigences réglementaires.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1033,21 +1045,9 @@
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:12:21.677249+00:00</t>
-        </is>
-      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Indicateur</t>
+          <t>Note de bas de page</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1083,14 +1083,14 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Risque opérationnel – Variation des niveaux de risque</t>
+          <t>Au cours du deuxième trimestre de 2025, la variation du risque opérationnel est liée à l’inclusion de CWB qui a été calculé selon l’approche standardisé conformément à l’approche utilisée par la Banque.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Risque opérationnel – Variation des niveaux de risque" a été ajouté dans le tableau de gestion du capital au T2 2025, alors qu'il était absent au T1 2025.
-Cet ajout permet de suivre plus précisément les variations des niveaux de risque opérationnel, ce qui est essentiel pour la gestion proactive des risques. Cela peut être en réponse à des exigences réglementaires ou à une volonté interne d'améliorer la surveillance des risques opérationnels.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier que cette nouvelle mesure est alignée avec les pratiques de gestion des risques opérationnels et qu'elle est conforme aux attentes des régulateurs.</t>
+          <t>La note de bas de page n-3 a été ajoutée dans le tableau de gestion du capital au T2 2025.
+Cette note précise que la variation du risque opérationnel est attribuée à l'inclusion de CWB, calculée selon l'approche standardisée. Cela indique un changement potentiel dans la manière dont le risque opérationnel est évalué, ce qui pourrait avoir des implications sur les ratios de capital réglementaire et la conformité aux normes de Bâle III.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette inclusion est cohérente avec les autres sections du rapport et vérifier si elle répond à de nouvelles exigences réglementaires.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1111,17 +1111,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Variation de l’actif pondéré en fonction des risques selon les principaux facteurs (1)</t>
+          <t>Variation des fonds propres réglementaires (1)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1137,14 +1137,14 @@
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Risque opérationnel – Méthode et politique</t>
+          <t>Émission d’actions ordinaires relatives à l'acquisition de CWB</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Risque opérationnel – Méthode et politique" a été ajouté dans le tableau de gestion du capital au T2 2025, alors qu'il était absent au T1 2025.
-Cet ajout reflète une approche plus détaillée dans la présentation des méthodes et politiques spécifiques au risque opérationnel. Cela peut indiquer une révision des politiques internes ou une réponse à des directives réglementaires exigeant une plus grande transparence dans la gestion des risques opérationnels.
-Il s'agit d'une mise à jour structurelle significative. L'analyste devrait confirmer que cette nouvelle présentation est cohérente avec les autres sections du rapport et qu'elle répond aux attentes des régulateurs.</t>
+          <t>L'indicateur "Émission d’actions ordinaires relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet indicateur n'était pas présent dans le trimestre précédent terminé le 31 janvier 2025.
+Cet ajout reflète une opération spécifique d'acquisition, ce qui peut avoir un impact significatif sur la structure du capital de la banque. Les émissions d'actions ordinaires dans le cadre d'acquisitions peuvent affecter les ratios de fonds propres, qui sont des éléments clés pour le respect des exigences réglementaires telles que Bâle III. Cela peut également influencer la perception des investisseurs et des régulateurs quant à la stratégie de croissance de la banque.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette émission est correctement intégrée dans les calculs des fonds propres et que les impacts sur les ratios réglementaires sont bien documentés.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1153,9 +1153,21 @@
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-23T18:58:47.043611+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1165,22 +1177,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Variation de l’actif pondéré en fonction des risques selon les principaux facteurs (1)</t>
+          <t>Variation des fonds propres réglementaires (1)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Note de bas de page</t>
+          <t>Indicateur</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1191,14 +1203,14 @@
       <c r="G13" s="2" t="inlineStr"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Au cours du deuxième trimestre de 2025, la variation du risque opérationnel est liée à l’inclusion de CWB qui a été calculé selon l’approche standardisé conformément à l’approche utilisée par la Banque.</t>
+          <t>Options de remplacement relatives à l'acquisition de CWB</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>La note de bas de page n-3 a été ajoutée dans le tableau de gestion du capital au T2 2025.
-Cette note précise que la variation du risque opérationnel est attribuée à l'inclusion de CWB, calculée selon l'approche standardisée. Cela indique un changement dans la composition du risque opérationnel, potentiellement lié à une acquisition ou à une intégration stratégique. Cette information est cruciale pour comprendre les ajustements dans le profil de risque de l'institution.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette inclusion est correctement reflétée dans les autres sections du rapport et qu'elle est conforme aux normes de divulgation et aux exigences réglementaires en matière de gestion des risques.</t>
+          <t>L'indicateur "Options de remplacement relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet indicateur n'était pas présent dans le trimestre précédent terminé le 31 janvier 2025.
+Cet ajout est lié à l'acquisition de CWB et concerne les options de remplacement, ce qui peut avoir des implications sur la valorisation des actions et les droits des actionnaires. Les options de remplacement peuvent modifier la structure du capital et influencer les calculs des fonds propres réglementaires, ce qui est crucial pour le respect des normes de Bâle III et des directives du BSIF.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier que ces options sont correctement évaluées et intégrées dans les rapports financiers, et que leur impact sur les ratios de fonds propres est bien compris.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1234,25 +1246,25 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Indicateur</t>
+          <t>Note de bas de page</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Émission d’actions ordinaires relatives à l'acquisition de CWB</t>
-        </is>
-      </c>
+          <t>Suppression</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Les données au 31 janvier 2025 tiennent compte du rachat d’actions privilégiées série 32 effectué le 17 février 2025.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Émission d’actions ordinaires relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet ajout reflète une opération spécifique liée à l'acquisition de CWB, ce qui n'était pas présent dans le trimestre précédent.
-L'ajout de cet indicateur est significatif car il met en lumière une transaction importante qui peut avoir un impact sur la structure du capital de la banque. Les émissions d'actions dans le cadre d'acquisitions peuvent affecter les ratios de fonds propres, qui sont des mesures clés suivies par les régulateurs tels que le BSIF dans le cadre des exigences de Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette émission est correctement intégrée dans les calculs des fonds propres et que les impacts sur les ratios prudentiels sont bien compris.</t>
+          <t>La note de bas de page n°2 a été supprimée du tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cette note était présente dans le trimestre précédent terminé le 31 janvier 2025.
+Cette note précisait que les données incluaient le rachat d’actions privilégiées série 32 effectué le 17 février 2025. La suppression de cette note pourrait indiquer que l'événement de rachat n'est plus pertinent pour la période actuelle ou que son impact a été entièrement intégré dans les chiffres présentés. Cela peut avoir des implications sur la transparence des informations fournies aux investisseurs et aux régulateurs, notamment en ce qui concerne la gestion des fonds propres et le respect des exigences de Bâle III.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que l'impact de ce rachat est correctement reflété dans les autres sections du rapport et que la suppression de la note ne compromet pas la compréhension des changements dans les fonds propres.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1273,342 +1285,138 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-19T00:12:11.271698+00:00</t>
+          <t>2026-04-23T18:58:52.570557+00:00</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Portefeuille d’actifs liquides (1)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Indicateur</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Suppression</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Actifs liquides – Au 31 janvier 2025</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>L'indicateur "Actifs liquides – Au 31 janvier 2025" a été retiré du tableau actuel, alors qu'il était présent dans le tableau précédent. Cet indicateur servait à fournir une référence temporelle spécifique pour les actifs liquides à une date antérieure, ce qui est une pratique courante pour contextualiser les données financières dans le temps.
+L'impact de cette suppression est principalement cosmétique, car elle ne modifie pas la méthodologie de calcul ou la présentation des actifs liquides eux-mêmes. Cependant, elle peut affecter la comparaison temporelle directe des données si les utilisateurs du rapport s'appuient sur ces dates pour suivre les tendances historiques. Dans le cadre des exigences réglementaires, cette suppression n'a pas d'incidence directe, car les dates de référence ne sont pas des éléments obligatoires de divulgation selon Bâle III ou les lignes directrices du BSIF.
+Il s'agit d'une mise à jour ordinaire visant probablement à simplifier la présentation du tableau. L'analyste devrait confirmer que les autres dates de référence pertinentes sont toujours présentes et que les utilisateurs du rapport ont accès à toutes les informations nécessaires pour une analyse temporelle complète.</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>analyst</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-23T18:58:56.509411+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Variation des fonds propres réglementaires (1)</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Indicateur</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Options de remplacement relatives à l'acquisition de CWB</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>L'indicateur "Options de remplacement relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet ajout est lié à l'acquisition de CWB et reflète des options de remplacement qui n'étaient pas présentes dans le trimestre précédent.
-Cet ajout est pertinent car il indique des ajustements spécifiques dans la structure du capital en raison de l'acquisition. Les options de remplacement peuvent influencer la composition des fonds propres et, par conséquent, les ratios de capital réglementaires. Ces ajustements doivent être conformes aux exigences de divulgation et de calcul des fonds propres selon les normes de Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier que ces options sont correctement comptabilisées et que leur impact sur les ratios de fonds propres est bien évalué.</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Indicateurs – Banques d’importance systémique mondiale (BISM) (1)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Suppression</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Indicateurs – Banques d’importance systémique mondiale (BISM) (1)</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Tableau supprimé du trimestre courant.</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr"/>
-      <c r="L15" s="2" t="inlineStr"/>
-      <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Variation des fonds propres réglementaires (1)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Note de bas de page</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Suppression</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Les données au 31 janvier 2025 tiennent compte du rachat d’actions privilégiées série 32 effectué le 17 février 2025.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>La note de bas de page n°2 a été supprimée dans le tableau des variations des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cette note faisait référence à l'impact du rachat d'actions privilégiées série 32 effectué le 17 février 2025, qui était pertinent pour le trimestre précédent.
-L'absence de cette note dans le rapport actuel pourrait indiquer que l'impact de ce rachat n'est plus pertinent pour la période actuelle ou que l'information a été intégrée ailleurs dans le rapport. Les rachats d'actions privilégiées peuvent affecter les fonds propres de catégorie 1 et, par conséquent, les ratios de capital réglementaires, qui sont surveillés de près par les régulateurs comme le BSIF dans le cadre des exigences de Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que l'impact de ce rachat est correctement reflété dans les calculs des fonds propres pour la période actuelle et que les ratios prudentiels sont toujours conformes aux exigences réglementaires.</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
-      <c r="L16" s="2" t="inlineStr"/>
-      <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Portefeuille d’actifs liquides (1)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Indicateur</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Au 30 avril 2025</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>Un nouvel en-tête de date 'Au 30 avril 2025' a été ajouté dans le tableau actuel. Cet en-tête semble être une simple mise à jour de la période de référence pour les données présentées dans le tableau des actifs liquides. Il est courant que les rapports financiers incluent des en-têtes de date pour indiquer la période couverte par les données.
-L'ajout de cet en-tête n'a pas d'impact direct sur les ratios prudentiels ou les exigences réglementaires, car il ne modifie pas la méthodologie de calcul ou la nature des indicateurs présentés. Il s'agit simplement d'une mise à jour de la période de référence, ce qui est une pratique standard dans les rapports financiers.
-Cet ajout est une mise à jour ordinaire et ne nécessite pas d'action particulière de la part de l'analyste. Il est recommandé de vérifier que les données associées à cette nouvelle période sont cohérentes avec les autres informations du rapport.</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>Validé</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>analyst</t>
         </is>
       </c>
-      <c r="N17" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-19T00:12:55.573736+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Portefeuille d’actifs liquides (1)</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>Indicateur</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Suppression</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Actifs liquides – Au 31 janvier 2025</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>L'en-tête de date 'Actifs liquides – Au 31 janvier 2025' a été supprimé du tableau précédent. Cette suppression semble être une mise à jour de la période de référence pour les données présentées dans le tableau des actifs liquides. Les en-têtes de date sont souvent utilisés pour indiquer la période couverte par les données dans les rapports financiers.
-La suppression de cet en-tête n'affecte pas directement les ratios prudentiels ou les exigences réglementaires, car elle ne modifie pas la méthodologie de calcul ou la nature des indicateurs présentés. Il s'agit simplement d'une mise à jour de la période de référence, ce qui est une pratique courante dans les rapports financiers.
-Cette suppression est une mise à jour ordinaire et ne nécessite pas d'action particulière de la part de l'analyste. Il est conseillé de s'assurer que les données pour la nouvelle période sont correctement reflétées dans le rapport.</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr"/>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Variation des fonds propres réglementaires (1)</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Indicateur</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Suppression</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Autres, y compris les ajustements réglementaires</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>L'indicateur "Autres, y compris les ajustements réglementaires" présent dans le tableau du trimestre terminé le 31 janvier 2025 a été supprimé dans le tableau du semestre terminé le 30 avril 2025. Cette suppression pourrait indiquer une réorganisation ou une clarification des ajustements réglementaires dans le tableau actuel.
-Bien que cet indicateur soit souvent utilisé pour regrouper divers ajustements mineurs, sa suppression pourrait refléter un changement dans la manière dont ces ajustements sont présentés ou calculés. Cela pourrait être lié à une mise à jour méthodologique ou à une simplification des divulgations.
-Il s'agit probablement d'une mise à jour cosmétique ou méthodologique. L'analyste devrait confirmer que les ajustements réglementaires sont toujours correctement reflétés dans d'autres parties du tableau ou du rapport.</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Indicateurs – Banques d’importance systémique mondiale (BISM) (1)</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Tableau</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Suppression</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Indicateurs – Banques d’importance systémique mondiale (BISM) (1)</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>Tableau supprimé du trimestre courant.</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="3" t="inlineStr"/>
-      <c r="N20" s="3" t="inlineStr"/>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-23T18:59:06.366153+00:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N20"/>
+  <autoFilter ref="A1:N16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Enhance AMF v2 integration tests and update justification requirements
- Updated justification texts for relevant and non-relevant changes to provide more context and clarity.
- Made justification mandatory for non-relevant changes, requiring a minimum of 200 characters and three sentences.
- Adjusted test cases to reflect changes in the justification logic and ensure compliance with new requirements.
- Enhanced filtering logic in the review queue to exclude non-relevant items and display relevant AMF fields correctly.
- Added integration tests for Dash components to verify proper rendering of AMF v2 fields and handling of non-relevant changes.
- Improved sorting logic in review items to prioritize categories and impacts correctly.
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changements détectés" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Changements détectés'!$A$1:$M$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -460,11 +460,10 @@
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -515,7 +514,7 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Nouvelle divulgation ?</t>
+          <t>Nouvelle idée ?</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -529,11 +528,6 @@
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Validé par</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Validé le</t>
         </is>
@@ -579,8 +573,8 @@
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>La note de bas de page n-1 a été ajoutée dans le tableau des échéances contractuelles des actifs financiers au T2 2025.
-Cette note précise l'impact de l'acquisition de CWB par la Banque, en indiquant que les résultats de CWB ont été consolidés à partir de la date de clôture, ce qui a affecté les soldes au 30 avril 2025. Cette information est cruciale car elle peut influencer la perception des investisseurs et des régulateurs sur la solidité financière de la Banque, notamment en ce qui concerne les ratios de capital et de liquidité. L'acquisition pourrait également avoir des implications sur les exigences de fonds propres selon les normes de Bâle III, en raison de l'intégration de nouveaux actifs et passifs.
-Il s'agit d'une divulgation importante qui pourrait avoir des implications structurelles sur l'analyse des états financiers de la Banque. L'analyste devrait confirmer l'intégration correcte de cette acquisition dans les autres sections du rapport financier et s'assurer que toutes les implications réglementaires ont été correctement adressées.</t>
+Cette note précise que la Banque a conclu l'acquisition de CWB le 3 février 2025, et que les résultats de CWB ont été consolidés à partir de cette date, impactant ainsi les soldes au 30 avril 2025. Cette information est cruciale car elle affecte directement la présentation des actifs financiers et pourrait influencer les ratios financiers et les analyses de risque associées.
+Il s'agit d'une divulgation importante liée à une acquisition stratégique. L'analyste devrait confirmer l'intégration correcte des résultats de CWB dans les états financiers consolidés et s'assurer que toutes les implications réglementaires et comptables ont été correctement adressées.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -591,7 +585,6 @@
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -633,19 +626,18 @@
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>L'indicateur "Risques émergents – Hausse et incertitude des droits de douane et des restrictions sur les échanges commerciaux" a été ajouté dans le tableau de gestion des risques au T2 2025, alors qu'il n'était pas présent au T1 2025.
-Cet ajout reflète une attention accrue aux risques liés aux fluctuations des droits de douane et aux restrictions commerciales, qui peuvent avoir un impact significatif sur les opérations bancaires internationales et la gestion des risques de crédit. Les institutions financières doivent surveiller ces évolutions pour ajuster leurs stratégies de couverture et de gestion des risques, conformément aux lignes directrices prudentielles.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cet ajout est aligné avec les autres sections du rapport sur les risques émergents et évaluer l'impact potentiel sur les stratégies de gestion des risques de l'institution.</t>
+Cet ajout reflète une attention accrue aux risques liés aux fluctuations des droits de douane et aux restrictions commerciales, qui peuvent avoir un impact significatif sur les opérations bancaires internationales et la gestion des risques de crédit. Les institutions financières doivent surveiller ces risques pour se conformer aux exigences réglementaires et maintenir la stabilité financière.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cet ajout est aligné avec les autres sections du rapport sur la gestion des risques et évaluer l'impact potentiel sur les stratégies de gestion des risques de l'institution.</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -687,19 +679,18 @@
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>L'indicateur "Risques émergents – Droits de douane sur les importations" a été retiré du tableau de gestion des risques au T2 2025, alors qu'il était présent au T1 2025.
-Ce retrait peut indiquer un changement dans la focalisation des risques émergents, passant d'une attention spécifique aux droits de douane sur les importations à une perspective plus large incluant les incertitudes et restrictions commerciales. Cela peut refléter une réévaluation des priorités en matière de gestion des risques, en réponse à des évolutions économiques ou politiques récentes.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier si ce retrait est compensé par d'autres indicateurs ou sections du rapport, et évaluer l'impact sur la stratégie globale de gestion des risques de l'institution.</t>
+Ce retrait peut indiquer un changement dans la focalisation des risques émergents, passant d'une attention spécifique aux droits de douane sur les importations à une perspective plus large englobant l'incertitude et les restrictions commerciales. Cela peut refléter une adaptation aux évolutions du contexte économique mondial et aux nouvelles directives réglementaires.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier si ce retrait est compensé par d'autres indicateurs ou sections du rapport et évaluer l'impact sur la communication des risques à l'interne et à l'externe.</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -742,30 +733,17 @@
         <is>
           <t>L'indicateur "Série 47" a été ajouté dans le tableau des actions privilégiées et autres instruments de capitaux propres au T2 2025, alors qu'il était absent au T1 2025.
 Cet ajout pourrait indiquer l'émission d'une nouvelle série d'actions privilégiées, ce qui peut avoir un impact sur la structure du capital de la banque. Les actions privilégiées sont souvent utilisées pour renforcer les fonds propres de catégorie 1, conformément aux exigences de Bâle III et aux lignes directrices du BSIF.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer l'émission de cette nouvelle série et s'assurer que les informations sont cohérentes avec les autres divulgations financières.</t>
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer l'émission de cette nouvelle série et évaluer son impact sur les ratios de fonds propres.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-23T18:57:41.194006+00:00</t>
-        </is>
-      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -807,19 +785,18 @@
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>L'indicateur "Série 49" a été ajouté dans le tableau des actions privilégiées et autres instruments de capitaux propres au T2 2025, alors qu'il était absent au T1 2025.
-L'ajout de cette série suggère une nouvelle émission d'actions privilégiées, ce qui peut influencer la composition des fonds propres de la banque. Les actions privilégiées jouent un rôle clé dans le renforcement des ratios de fonds propres, en ligne avec les exigences réglementaires de Bâle III.
-Il s'agit d'une mise à jour structurelle significative. L'analyste devrait vérifier l'exactitude de cette nouvelle émission et son impact sur les ratios de fonds propres.</t>
+Cet ajout pourrait indiquer l'émission d'une nouvelle série d'actions privilégiées, ce qui peut avoir un impact sur la structure du capital de la banque. Les actions privilégiées sont souvent utilisées pour renforcer les fonds propres de catégorie 1, conformément aux exigences de Bâle III et aux lignes directrices du BSIF.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer l'émission de cette nouvelle série et évaluer son impact sur les ratios de fonds propres.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -861,19 +838,18 @@
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>L'indicateur "Série 32" a été retiré du tableau des actions privilégiées et autres instruments de capitaux propres au T2 2025, alors qu'il était présent au T1 2025.
-La suppression de cette série peut indiquer le rachat ou l'annulation de cette émission d'actions privilégiées, ce qui pourrait affecter la structure du capital de la banque. Les actions privilégiées sont essentielles pour maintenir les ratios de fonds propres requis par Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer la raison de cette suppression et évaluer son impact sur les ratios de fonds propres et la conformité réglementaire.</t>
+La suppression de cette série pourrait indiquer le rachat ou l'annulation de cette série d'actions privilégiées, ce qui peut affecter la composition des fonds propres de la banque. Cela pourrait avoir des implications sur les ratios de fonds propres, notamment ceux liés aux exigences de Bâle III.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier les raisons de cette suppression et évaluer son impact sur la structure du capital.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -914,32 +890,19 @@
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>La note de bas de page n°3 a été supprimée dans le tableau de gestion du capital réglementaire, du ratio de levier et du TLAC. Cette note faisait référence à l'impact du rachat d'actions privilégiées série 32 sur les données au 31 janvier 2025.
-L'absence de cette note dans le rapport actuel pourrait indiquer que l'effet de ce rachat n'est plus pertinent pour la période actuelle ou que l'information a été intégrée ailleurs dans le rapport. Cela pourrait avoir un impact sur la compréhension des ajustements de capital et des ratios de fonds propres, notamment si ces ajustements influencent les calculs de Bâle III ou les exigences du BSIF.
-Il s'agit potentiellement d'une mise à jour structurelle. L'analyste devrait confirmer si l'impact du rachat d'actions a été traité différemment dans le rapport actuel ou s'il est devenu obsolète. Une vérification de la cohérence avec d'autres sections du rapport est recommandée.</t>
+          <t>La note de bas de page n°3 a été supprimée du tableau de gestion du capital réglementaire, du ratio de levier et du TLAC dans le rapport du T2 2025. Cette note indiquait que les données au 31 janvier 2025 prenaient en compte le rachat d’actions privilégiées série 32 effectué le 17 février 2025.
+L'absence de cette note dans le rapport actuel pourrait avoir des implications sur la transparence des informations fournies aux investisseurs et aux régulateurs. Le rachat d'actions privilégiées peut affecter les fonds propres de catégorie 1 et, par conséquent, les ratios de capital réglementaire. Selon les lignes directrices de Bâle III et les exigences du BSIF, toute modification significative des fonds propres doit être clairement divulguée pour assurer la conformité réglementaire et la transparence.
+Il s'agit d'une mise à jour structurelle qui nécessite une vérification pour s'assurer que l'impact du rachat d'actions est toujours correctement reflété dans les données financières présentées. L'analyste devrait confirmer que l'absence de cette note n'entraîne pas de malentendu sur les chiffres rapportés et que les informations pertinentes sont intégrées ailleurs dans le rapport.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-23T18:59:00.240659+00:00</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -980,20 +943,19 @@
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>La note de bas de page n°4 a été supprimée dans le tableau des exigences réglementaires de ratios des fonds propres, de levier et TLAC au T2 2025. Cette note indiquait que les ratios au 31 janvier 2025 prenaient en compte le rachat d’actions privilégiées série 32 effectué le 17 février 2025.
-L'absence de cette note dans le rapport actuel pourrait avoir un impact sur la transparence des informations fournies aux investisseurs et aux régulateurs. En effet, le rachat d'actions privilégiées peut influencer les ratios de fonds propres, et son omission pourrait masquer des variations importantes dans les calculs des ratios prudentiels. Selon les lignes directrices du BSIF, toute modification significative des éléments de fonds propres doit être clairement divulguée pour assurer la conformité avec les exigences de Bâle III.
-Il s'agit d'une mise à jour potentiellement significative qui pourrait indiquer un changement dans la manière dont les événements postérieurs sont pris en compte dans les calculs des ratios. L'analyste devrait confirmer si cette omission est intentionnelle et si elle est conforme aux pratiques de divulgation actuelles. Une investigation plus approfondie est recommandée pour s'assurer que toutes les informations pertinentes sont correctement communiquées.</t>
+          <t>La note de bas de page n-4 a été supprimée dans le tableau des exigences réglementaires de ratios des fonds propres, de levier et TLAC au T2 2025.
+Cette note indiquait que les ratios au 31 janvier 2025 prenaient en compte le rachat d’actions privilégiées série 32 effectué le 17 février 2025. La suppression de cette note pourrait indiquer que l'impact de ce rachat n'est plus pertinent pour les ratios actuels ou que l'information a été intégrée ailleurs dans le rapport.
+Il s'agit d'une mise à jour potentiellement significative, car elle pourrait affecter la compréhension des ajustements des ratios de fonds propres. L'analyste devrait confirmer si cette information est redondante ou si elle a été déplacée, et s'assurer que la transparence des divulgations est maintenue.</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1018,7 +980,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Indicateur</t>
+          <t>Note de bas de page</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1029,25 +991,24 @@
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Risque de marché – Acquisitions et cessions</t>
+          <t>Au cours du deuxième trimestre de 2025, la variation du risque opérationnel est liée à l’inclusion de CWB qui a été calculé selon l’approche standardisé conformément à l’approche utilisée par la Banque.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Risque de marché – Acquisitions et cessions" a été ajouté dans le tableau de gestion du capital au T2 2025, alors qu'il était absent au T1 2025.
-Cet ajout permet de mieux isoler l'impact des acquisitions et cessions sur le risque de marché, ce qui est crucial pour l'évaluation des risques et la planification stratégique. Cela pourrait être lié à des changements dans la structure de l'entreprise ou à des exigences de divulgation accrues.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait s'assurer que cette nouvelle catégorie est justifiée par des changements dans les opérations ou les exigences réglementaires.</t>
+          <t>La note de bas de page n-3 a été ajoutée dans le tableau de gestion du capital au T2 2025.
+Cette note précise que la variation du risque opérationnel est due à l'inclusion de CWB, calculée selon l'approche standardisée. Cela indique un changement dans la composition du risque opérationnel, potentiellement lié à une acquisition ou une intégration stratégique. L'approche standardisée est conforme aux pratiques de Bâle III, ce qui peut influencer les exigences en capital et la gestion des risques.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que l'inclusion de CWB est correctement intégrée dans les calculs de risque et que les divulgations sont cohérentes avec les autres sections du rapport.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1057,22 +1018,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Variation de l’actif pondéré en fonction des risques selon les principaux facteurs (1)</t>
+          <t>Variation des fonds propres réglementaires (1)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Note de bas de page</t>
+          <t>Indicateur</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1083,25 +1044,24 @@
       <c r="G11" s="2" t="inlineStr"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Au cours du deuxième trimestre de 2025, la variation du risque opérationnel est liée à l’inclusion de CWB qui a été calculé selon l’approche standardisé conformément à l’approche utilisée par la Banque.</t>
+          <t>Émission d’actions ordinaires relatives à l'acquisition de CWB</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>La note de bas de page n-3 a été ajoutée dans le tableau de gestion du capital au T2 2025.
-Cette note précise que la variation du risque opérationnel est attribuée à l'inclusion de CWB, calculée selon l'approche standardisée. Cela indique un changement potentiel dans la manière dont le risque opérationnel est évalué, ce qui pourrait avoir des implications sur les ratios de capital réglementaire et la conformité aux normes de Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette inclusion est cohérente avec les autres sections du rapport et vérifier si elle répond à de nouvelles exigences réglementaires.</t>
+          <t>L'indicateur "Émission d’actions ordinaires relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet indicateur n'était pas présent dans le trimestre précédent terminé le 31 janvier 2025.
+Cet ajout reflète une opération spécifique d'émission d'actions ordinaires liée à l'acquisition de CWB. Cela peut avoir un impact significatif sur la structure du capital de la banque, influençant potentiellement les ratios de fonds propres réglementaires tels que le CET1. Les exigences de Bâle III et les lignes directrices du BSIF sur la divulgation des fonds propres pourraient être concernées, car elles nécessitent une transparence accrue sur les événements affectant les fonds propres.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette émission est correctement intégrée dans les calculs des fonds propres et que toutes les implications réglementaires sont bien prises en compte.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1137,37 +1097,24 @@
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Émission d’actions ordinaires relatives à l'acquisition de CWB</t>
+          <t>Options de remplacement relatives à l'acquisition de CWB</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Émission d’actions ordinaires relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet indicateur n'était pas présent dans le trimestre précédent terminé le 31 janvier 2025.
-Cet ajout reflète une opération spécifique d'acquisition, ce qui peut avoir un impact significatif sur la structure du capital de la banque. Les émissions d'actions ordinaires dans le cadre d'acquisitions peuvent affecter les ratios de fonds propres, qui sont des éléments clés pour le respect des exigences réglementaires telles que Bâle III. Cela peut également influencer la perception des investisseurs et des régulateurs quant à la stratégie de croissance de la banque.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que cette émission est correctement intégrée dans les calculs des fonds propres et que les impacts sur les ratios réglementaires sont bien documentés.</t>
+          <t>L'indicateur "Options de remplacement relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet indicateur n'était pas présent dans le trimestre précédent terminé le 31 janvier 2025.
+Cet ajout indique que des options de remplacement ont été émises dans le cadre de l'acquisition de CWB. Cela peut affecter la valorisation des actions et les calculs des fonds propres, influençant potentiellement les ratios de fonds propres réglementaires. Les exigences de Bâle III et les lignes directrices du BSIF sur la divulgation des fonds propres pourraient être concernées, car elles nécessitent une transparence accrue sur les événements affectant les fonds propres.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier que ces options sont correctement intégrées dans les calculs des fonds propres et que toutes les implications réglementaires sont bien prises en compte.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-23T18:58:47.043611+00:00</t>
-        </is>
-      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1192,231 +1139,85 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Indicateur</t>
+          <t>Note de bas de page</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Options de remplacement relatives à l'acquisition de CWB</t>
-        </is>
-      </c>
+          <t>Suppression</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Les données au 31 janvier 2025 tiennent compte du rachat d’actions privilégiées série 32 effectué le 17 février 2025.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>L'indicateur "Options de remplacement relatives à l'acquisition de CWB" a été ajouté dans le tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cet indicateur n'était pas présent dans le trimestre précédent terminé le 31 janvier 2025.
-Cet ajout est lié à l'acquisition de CWB et concerne les options de remplacement, ce qui peut avoir des implications sur la valorisation des actions et les droits des actionnaires. Les options de remplacement peuvent modifier la structure du capital et influencer les calculs des fonds propres réglementaires, ce qui est crucial pour le respect des normes de Bâle III et des directives du BSIF.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait vérifier que ces options sont correctement évaluées et intégrées dans les rapports financiers, et que leur impact sur les ratios de fonds propres est bien compris.</t>
+          <t>La note de bas de page n°2 a été supprimée du tableau des variations des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cette note indiquait que les données au 31 janvier 2025 prenaient en compte le rachat d’actions privilégiées série 32 effectué le 17 février 2025.
+La suppression de cette note pourrait avoir un impact sur la transparence des informations fournies aux investisseurs et aux régulateurs concernant les événements affectant les fonds propres de la banque. Le rachat d'actions privilégiées peut influencer les ratios de fonds propres réglementaires, tels que le CET1, et doit être correctement divulgué conformément aux exigences de Bâle III et aux lignes directrices du BSIF.
+Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que l'impact de ce rachat est toujours correctement intégré dans les calculs des fonds propres et que toutes les implications réglementaires sont bien prises en compte. Une vérification supplémentaire pourrait être nécessaire pour s'assurer que cette information n'est pas omise ailleurs dans le rapport.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Variation des fonds propres réglementaires (1)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Note de bas de page</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Indicateurs – Banques d’importance systémique mondiale (BISM) (1)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Tableau</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Suppression</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Les données au 31 janvier 2025 tiennent compte du rachat d’actions privilégiées série 32 effectué le 17 février 2025.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>La note de bas de page n°2 a été supprimée du tableau de variation des fonds propres réglementaires pour le semestre terminé le 30 avril 2025. Cette note était présente dans le trimestre précédent terminé le 31 janvier 2025.
-Cette note précisait que les données incluaient le rachat d’actions privilégiées série 32 effectué le 17 février 2025. La suppression de cette note pourrait indiquer que l'événement de rachat n'est plus pertinent pour la période actuelle ou que son impact a été entièrement intégré dans les chiffres présentés. Cela peut avoir des implications sur la transparence des informations fournies aux investisseurs et aux régulateurs, notamment en ce qui concerne la gestion des fonds propres et le respect des exigences de Bâle III.
-Il s'agit d'une mise à jour structurelle importante. L'analyste devrait confirmer que l'impact de ce rachat est correctement reflété dans les autres sections du rapport et que la suppression de la note ne compromet pas la compréhension des changements dans les fonds propres.</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-23T18:58:52.570557+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Portefeuille d’actifs liquides (1)</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>37</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Indicateur</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Suppression</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Actifs liquides – Au 31 janvier 2025</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>L'indicateur "Actifs liquides – Au 31 janvier 2025" a été retiré du tableau actuel, alors qu'il était présent dans le tableau précédent. Cet indicateur servait à fournir une référence temporelle spécifique pour les actifs liquides à une date antérieure, ce qui est une pratique courante pour contextualiser les données financières dans le temps.
-L'impact de cette suppression est principalement cosmétique, car elle ne modifie pas la méthodologie de calcul ou la présentation des actifs liquides eux-mêmes. Cependant, elle peut affecter la comparaison temporelle directe des données si les utilisateurs du rapport s'appuient sur ces dates pour suivre les tendances historiques. Dans le cadre des exigences réglementaires, cette suppression n'a pas d'incidence directe, car les dates de référence ne sont pas des éléments obligatoires de divulgation selon Bâle III ou les lignes directrices du BSIF.
-Il s'agit d'une mise à jour ordinaire visant probablement à simplifier la présentation du tableau. L'analyste devrait confirmer que les autres dates de référence pertinentes sont toujours présentes et que les utilisateurs du rapport ont accès à toutes les informations nécessaires pour une analyse temporelle complète.</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M15" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N15" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-23T18:58:56.509411+00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Indicateurs – Banques d’importance systémique mondiale (BISM) (1)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>Tableau</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Suppression</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Indicateurs – Banques d’importance systémique mondiale (BISM) (1)</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>Tableau supprimé du trimestre courant.</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M16" s="3" t="inlineStr">
-        <is>
-          <t>analyst</t>
-        </is>
-      </c>
-      <c r="N16" s="3" t="inlineStr">
-        <is>
-          <t>2026-04-23T18:59:06.366153+00:00</t>
-        </is>
-      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>OUI, le retrait du tableau 'Indicateurs – Banques d’importance systémique mondiale (BISM)' est substantiel. Ce tableau contenait des indicateurs clés tels que l'activité transfrontière, la taille, l'interdépendance, la substituabilité/infrastructure financière et la complexité. Ces indicateurs sont cruciaux pour évaluer l'importance systémique d'une banque. Leur suppression modifie la structure du rapport et la divulgation des risques associés aux BISM. Cela représente un changement significatif dans la manière dont la banque communique ses risques systémiques, ce qui est pertinent pour les thèmes AMF de DIVULGATION_RETRAIT et STRUCTURE_RAPPORT.</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N16"/>
+  <autoFilter ref="A1:M14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add T4 section localization support
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-11T14:00:39.880382+00:00</t>
+          <t>2026-06-23T15:19:10.056827+00:00</t>
         </is>
       </c>
     </row>
@@ -793,16 +793,8 @@
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-11T14:00:40.430625+00:00</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add change segment support and update BNC text comparison outputs
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -581,8 +581,16 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T19:42:33.142071+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -741,7 +749,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23T15:19:10.056827+00:00</t>
+          <t>2026-06-24T19:42:25.262918+00:00</t>
         </is>
       </c>
     </row>
@@ -793,8 +801,16 @@
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T19:42:55.559989+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1048,8 +1064,16 @@
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
-      <c r="M11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24T19:42:57.806568+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add visual proof zoom modal
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -581,16 +581,8 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-24T19:42:33.142071+00:00</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -749,7 +741,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T19:42:25.262918+00:00</t>
+          <t>2026-06-25T15:17:25.021843+00:00</t>
         </is>
       </c>
     </row>
@@ -808,7 +800,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T19:42:55.559989+00:00</t>
+          <t>2026-06-25T15:19:11.366220+00:00</t>
         </is>
       </c>
     </row>
@@ -911,8 +903,16 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T15:19:18.162270+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -962,8 +962,16 @@
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25T15:19:19.751155+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1071,7 +1079,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-24T19:42:57.806568+00:00</t>
+          <t>2026-06-25T15:17:57.233229+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(text-analysis): deduplicate block comparisons and group page numbers in text_comparison.json and outputs
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -479,12 +479,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Page T1</t>
+          <t>Page (trimestre précédent)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Page T2</t>
+          <t>Page (trimestre courant)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -499,12 +499,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Libellé T1</t>
+          <t>Libellé (trimestre précédent)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Libellé T2</t>
+          <t>Libellé (trimestre courant)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -581,8 +581,16 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-28T03:59:55.662559+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -741,7 +749,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25T15:17:25.021843+00:00</t>
+          <t>2026-07-28T03:57:01.038922+00:00</t>
         </is>
       </c>
     </row>
@@ -793,16 +801,8 @@
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-25T15:19:11.366220+00:00</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25T15:19:18.162270+00:00</t>
+          <t>2026-07-28T03:59:45.951819+00:00</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25T15:19:19.751155+00:00</t>
+          <t>2026-07-28T03:59:28.404628+00:00</t>
         </is>
       </c>
     </row>
@@ -1072,16 +1072,8 @@
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-25T15:17:57.233229+00:00</t>
-        </is>
-      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
refactor: remove legacy src/vigilance/extract directory and obsolete prototype tests
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -581,16 +581,8 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-28T03:59:55.662559+00:00</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -749,7 +741,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28T03:57:01.038922+00:00</t>
+          <t>2026-07-30T18:40:54.988811+00:00</t>
         </is>
       </c>
     </row>
@@ -903,16 +895,8 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-28T03:59:45.951819+00:00</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -962,16 +946,8 @@
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-28T03:59:28.404628+00:00</t>
-        </is>
-      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data(validation): publish latest analyst artifacts
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/comparison.xlsx
@@ -734,16 +734,8 @@
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Validé</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-30T18:40:54.988811+00:00</t>
-        </is>
-      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1197,8 +1189,16 @@
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07T05:53:34.016117+00:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M14"/>

</xml_diff>